<commit_message>
Updating Module 1 and HW 1 for 2026
</commit_message>
<xml_diff>
--- a/book/modules/data/Skykomish_peak_flow_12134500_WY1929_2025.xlsx
+++ b/book/modules/data/Skykomish_peak_flow_12134500_WY1929_2025.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jdlund/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B49FB02F-0B8C-CF41-9F2E-02C3A098D5FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD9B8EEE-2AA0-3A46-812F-FB8D735DA270}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17880" yWindow="-16960" windowWidth="25040" windowHeight="15740" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-2320" yWindow="-20920" windowWidth="25040" windowHeight="15740" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="peak_flow_12134500_skykomish_ri" sheetId="1" r:id="rId1"/>
@@ -424,7 +424,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D97"/>
+  <dimension ref="A1:D98"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="10.83203125" style="2"/>
@@ -1657,211 +1657,225 @@
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A83" s="1">
-        <v>40560</v>
+        <v>40117</v>
       </c>
       <c r="B83" s="2">
-        <v>2011</v>
+        <v>2010</v>
       </c>
       <c r="C83">
-        <v>63900</v>
+        <v>27800</v>
       </c>
       <c r="D83">
-        <v>18.36</v>
+        <v>13.23</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A84" s="1">
-        <v>40905</v>
+        <v>40560</v>
       </c>
       <c r="B84" s="2">
-        <v>2012</v>
+        <v>2011</v>
       </c>
       <c r="C84">
-        <v>25300</v>
+        <v>63900</v>
       </c>
       <c r="D84">
-        <v>12.76</v>
+        <v>18.36</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A85" s="1">
-        <v>41211</v>
+        <v>40905</v>
       </c>
       <c r="B85" s="2">
-        <v>2013</v>
+        <v>2012</v>
       </c>
       <c r="C85">
-        <v>26800</v>
+        <v>25300</v>
       </c>
       <c r="D85">
-        <v>13.05</v>
+        <v>12.76</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A86" s="1">
-        <v>41707</v>
+        <v>41211</v>
       </c>
       <c r="B86" s="2">
-        <v>2014</v>
+        <v>2013</v>
       </c>
       <c r="C86">
-        <v>38900</v>
+        <v>26800</v>
       </c>
       <c r="D86">
-        <v>15.08</v>
+        <v>13.05</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A87" s="1">
-        <v>41971</v>
+        <v>41707</v>
       </c>
       <c r="B87" s="2">
-        <v>2015</v>
+        <v>2014</v>
       </c>
       <c r="C87">
-        <v>58100</v>
+        <v>38900</v>
       </c>
       <c r="D87">
-        <v>17.670000000000002</v>
+        <v>15.08</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A88" s="1">
-        <v>42325</v>
+        <v>41971</v>
       </c>
       <c r="B88" s="2">
-        <v>2016</v>
+        <v>2015</v>
       </c>
       <c r="C88">
-        <v>95900</v>
+        <v>58100</v>
       </c>
       <c r="D88">
-        <v>21.73</v>
+        <v>17.670000000000002</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A89" s="1">
-        <v>42663</v>
+        <v>42325</v>
       </c>
       <c r="B89" s="2">
-        <v>2017</v>
+        <v>2016</v>
       </c>
       <c r="C89">
-        <v>41000</v>
+        <v>95900</v>
       </c>
       <c r="D89">
-        <v>15.76</v>
+        <v>21.73</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A90" s="1">
-        <v>43062</v>
+        <v>42663</v>
       </c>
       <c r="B90" s="2">
-        <v>2018</v>
+        <v>2017</v>
       </c>
       <c r="C90">
-        <v>54200</v>
+        <v>41000</v>
       </c>
       <c r="D90">
-        <v>17.5</v>
+        <v>15.76</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A91" s="1">
-        <v>43406</v>
+        <v>43062</v>
       </c>
       <c r="B91" s="2">
-        <v>2019</v>
+        <v>2018</v>
       </c>
       <c r="C91">
-        <v>35200</v>
+        <v>54200</v>
       </c>
       <c r="D91">
-        <v>14.98</v>
+        <v>17.5</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A92" s="1">
-        <v>43862</v>
+        <v>43406</v>
       </c>
       <c r="B92" s="2">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="C92">
-        <v>72200</v>
+        <v>35200</v>
       </c>
       <c r="D92">
-        <v>19.5</v>
+        <v>14.98</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A93" s="1">
-        <v>44209</v>
+        <v>43862</v>
       </c>
       <c r="B93" s="2">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C93">
-        <v>37400</v>
+        <v>72200</v>
       </c>
       <c r="D93">
-        <v>15.26</v>
+        <v>19.5</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A94" s="1">
-        <v>44514</v>
+        <v>44209</v>
       </c>
       <c r="B94" s="2">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C94">
-        <v>57900</v>
+        <v>37400</v>
       </c>
       <c r="D94">
-        <v>17.940000000000001</v>
+        <v>15.26</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A95" s="1">
-        <v>44870</v>
+        <v>44514</v>
       </c>
       <c r="B95" s="2">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C95">
-        <v>53300</v>
+        <v>57900</v>
       </c>
       <c r="D95">
-        <v>17.41</v>
+        <v>17.940000000000001</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A96" s="1">
-        <v>45265</v>
+        <v>44870</v>
       </c>
       <c r="B96" s="2">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C96">
-        <v>58300</v>
+        <v>53300</v>
       </c>
       <c r="D96">
-        <v>17.989999999999998</v>
+        <v>17.41</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A97" s="1">
+        <v>45265</v>
+      </c>
+      <c r="B97" s="2">
+        <v>2024</v>
+      </c>
+      <c r="C97">
+        <v>58300</v>
+      </c>
+      <c r="D97">
+        <v>17.989999999999998</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A98" s="1">
         <v>45740</v>
       </c>
-      <c r="B97" s="2">
+      <c r="B98" s="2">
         <v>2025</v>
       </c>
-      <c r="C97">
+      <c r="C98">
         <v>30900</v>
       </c>
-      <c r="D97">
+      <c r="D98">
         <v>14.68</v>
       </c>
     </row>

</xml_diff>